<commit_message>
Fix date formatting and add natural gas feature engineering
</commit_message>
<xml_diff>
--- a/linear_regression/cleaned_data/nat_gas_consume_cleaned.xlsx
+++ b/linear_regression/cleaned_data/nat_gas_consume_cleaned.xlsx
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>01-01-2001</t>
+          <t>2001-01-01</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -453,7 +453,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>01-02-2001</t>
+          <t>2001-02-01</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -463,7 +463,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>01-03-2001</t>
+          <t>2001-03-01</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -473,7 +473,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>01-04-2001</t>
+          <t>2001-04-01</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -483,7 +483,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01-05-2001</t>
+          <t>2001-05-01</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -493,7 +493,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01-06-2001</t>
+          <t>2001-06-01</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -503,7 +503,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>01-07-2001</t>
+          <t>2001-07-01</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -513,7 +513,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>01-08-2001</t>
+          <t>2001-08-01</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -523,7 +523,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>01-09-2001</t>
+          <t>2001-09-01</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -533,7 +533,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>01-10-2001</t>
+          <t>2001-10-01</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -543,7 +543,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>01-11-2001</t>
+          <t>2001-11-01</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -553,7 +553,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>01-12-2001</t>
+          <t>2001-12-01</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -563,7 +563,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>01-01-2002</t>
+          <t>2002-01-01</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -573,7 +573,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>01-02-2002</t>
+          <t>2002-02-01</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -583,7 +583,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>01-03-2002</t>
+          <t>2002-03-01</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -593,7 +593,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>01-04-2002</t>
+          <t>2002-04-01</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -603,7 +603,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>01-05-2002</t>
+          <t>2002-05-01</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -613,7 +613,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>01-06-2002</t>
+          <t>2002-06-01</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -623,7 +623,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>01-07-2002</t>
+          <t>2002-07-01</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -633,7 +633,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>01-08-2002</t>
+          <t>2002-08-01</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -643,7 +643,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>01-09-2002</t>
+          <t>2002-09-01</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -653,7 +653,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>01-10-2002</t>
+          <t>2002-10-01</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -663,7 +663,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>01-11-2002</t>
+          <t>2002-11-01</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -673,7 +673,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>01-12-2002</t>
+          <t>2002-12-01</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -683,7 +683,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>01-01-2003</t>
+          <t>2003-01-01</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -693,7 +693,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>01-02-2003</t>
+          <t>2003-02-01</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -703,7 +703,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>01-03-2003</t>
+          <t>2003-03-01</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -713,7 +713,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>01-04-2003</t>
+          <t>2003-04-01</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -723,7 +723,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>01-05-2003</t>
+          <t>2003-05-01</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -733,7 +733,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>01-06-2003</t>
+          <t>2003-06-01</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -743,7 +743,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>01-07-2003</t>
+          <t>2003-07-01</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -753,7 +753,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>01-08-2003</t>
+          <t>2003-08-01</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -763,7 +763,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>01-09-2003</t>
+          <t>2003-09-01</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -773,7 +773,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>01-10-2003</t>
+          <t>2003-10-01</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -783,7 +783,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>01-11-2003</t>
+          <t>2003-11-01</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -793,7 +793,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>01-12-2003</t>
+          <t>2003-12-01</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -803,7 +803,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>01-01-2004</t>
+          <t>2004-01-01</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -813,7 +813,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>01-02-2004</t>
+          <t>2004-02-01</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -823,7 +823,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>01-03-2004</t>
+          <t>2004-03-01</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -833,7 +833,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>01-04-2004</t>
+          <t>2004-04-01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -843,7 +843,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>01-05-2004</t>
+          <t>2004-05-01</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -853,7 +853,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>01-06-2004</t>
+          <t>2004-06-01</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -863,7 +863,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>01-07-2004</t>
+          <t>2004-07-01</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -873,7 +873,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>01-08-2004</t>
+          <t>2004-08-01</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -883,7 +883,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>01-09-2004</t>
+          <t>2004-09-01</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -893,7 +893,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>01-10-2004</t>
+          <t>2004-10-01</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -903,7 +903,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>01-11-2004</t>
+          <t>2004-11-01</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -913,7 +913,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>01-12-2004</t>
+          <t>2004-12-01</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -923,7 +923,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>01-01-2005</t>
+          <t>2005-01-01</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -933,7 +933,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>01-02-2005</t>
+          <t>2005-02-01</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -943,7 +943,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>01-03-2005</t>
+          <t>2005-03-01</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -953,7 +953,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>01-04-2005</t>
+          <t>2005-04-01</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -963,7 +963,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>01-05-2005</t>
+          <t>2005-05-01</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -973,7 +973,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>01-06-2005</t>
+          <t>2005-06-01</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -983,7 +983,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>01-07-2005</t>
+          <t>2005-07-01</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -993,7 +993,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>01-08-2005</t>
+          <t>2005-08-01</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1003,7 +1003,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>01-09-2005</t>
+          <t>2005-09-01</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1013,7 +1013,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>01-10-2005</t>
+          <t>2005-10-01</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1023,7 +1023,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>01-11-2005</t>
+          <t>2005-11-01</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1033,7 +1033,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>01-12-2005</t>
+          <t>2005-12-01</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1043,7 +1043,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>01-01-2006</t>
+          <t>2006-01-01</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1053,7 +1053,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>01-02-2006</t>
+          <t>2006-02-01</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1063,7 +1063,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>01-03-2006</t>
+          <t>2006-03-01</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1073,7 +1073,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>01-04-2006</t>
+          <t>2006-04-01</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1083,7 +1083,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>01-05-2006</t>
+          <t>2006-05-01</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1093,7 +1093,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>01-06-2006</t>
+          <t>2006-06-01</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1103,7 +1103,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>01-07-2006</t>
+          <t>2006-07-01</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1113,7 +1113,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>01-08-2006</t>
+          <t>2006-08-01</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1123,7 +1123,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>01-09-2006</t>
+          <t>2006-09-01</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1133,7 +1133,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>01-10-2006</t>
+          <t>2006-10-01</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1143,7 +1143,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>01-11-2006</t>
+          <t>2006-11-01</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1153,7 +1153,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>01-12-2006</t>
+          <t>2006-12-01</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1163,7 +1163,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>01-01-2007</t>
+          <t>2007-01-01</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1173,7 +1173,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>01-02-2007</t>
+          <t>2007-02-01</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1183,7 +1183,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>01-03-2007</t>
+          <t>2007-03-01</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1193,7 +1193,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>01-04-2007</t>
+          <t>2007-04-01</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1203,7 +1203,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>01-05-2007</t>
+          <t>2007-05-01</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1213,7 +1213,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>01-06-2007</t>
+          <t>2007-06-01</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1223,7 +1223,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>01-07-2007</t>
+          <t>2007-07-01</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1233,7 +1233,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>01-08-2007</t>
+          <t>2007-08-01</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1243,7 +1243,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>01-09-2007</t>
+          <t>2007-09-01</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1253,7 +1253,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>01-10-2007</t>
+          <t>2007-10-01</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1263,7 +1263,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>01-11-2007</t>
+          <t>2007-11-01</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1273,7 +1273,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>01-12-2007</t>
+          <t>2007-12-01</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1283,7 +1283,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>01-01-2008</t>
+          <t>2008-01-01</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1293,7 +1293,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>01-02-2008</t>
+          <t>2008-02-01</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1303,7 +1303,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>01-03-2008</t>
+          <t>2008-03-01</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1313,7 +1313,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>01-04-2008</t>
+          <t>2008-04-01</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1323,7 +1323,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>01-05-2008</t>
+          <t>2008-05-01</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1333,7 +1333,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>01-06-2008</t>
+          <t>2008-06-01</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1343,7 +1343,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>01-07-2008</t>
+          <t>2008-07-01</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1353,7 +1353,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>01-08-2008</t>
+          <t>2008-08-01</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1363,7 +1363,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>01-09-2008</t>
+          <t>2008-09-01</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1373,7 +1373,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>01-10-2008</t>
+          <t>2008-10-01</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1383,7 +1383,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>01-11-2008</t>
+          <t>2008-11-01</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1393,7 +1393,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>01-12-2008</t>
+          <t>2008-12-01</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1403,7 +1403,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>01-01-2009</t>
+          <t>2009-01-01</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1413,7 +1413,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>01-02-2009</t>
+          <t>2009-02-01</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -1423,7 +1423,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>01-03-2009</t>
+          <t>2009-03-01</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -1433,7 +1433,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>01-04-2009</t>
+          <t>2009-04-01</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -1443,7 +1443,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>01-05-2009</t>
+          <t>2009-05-01</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -1453,7 +1453,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>01-06-2009</t>
+          <t>2009-06-01</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -1463,7 +1463,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>01-07-2009</t>
+          <t>2009-07-01</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -1473,7 +1473,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>01-08-2009</t>
+          <t>2009-08-01</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -1483,7 +1483,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>01-09-2009</t>
+          <t>2009-09-01</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -1493,7 +1493,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>01-10-2009</t>
+          <t>2009-10-01</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -1503,7 +1503,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>01-11-2009</t>
+          <t>2009-11-01</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -1513,7 +1513,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>01-12-2009</t>
+          <t>2009-12-01</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -1523,7 +1523,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>01-01-2010</t>
+          <t>2010-01-01</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -1533,7 +1533,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>01-02-2010</t>
+          <t>2010-02-01</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -1543,7 +1543,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>01-03-2010</t>
+          <t>2010-03-01</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -1553,7 +1553,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>01-04-2010</t>
+          <t>2010-04-01</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -1563,7 +1563,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>01-05-2010</t>
+          <t>2010-05-01</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -1573,7 +1573,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>01-06-2010</t>
+          <t>2010-06-01</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -1583,7 +1583,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>01-07-2010</t>
+          <t>2010-07-01</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -1593,7 +1593,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>01-08-2010</t>
+          <t>2010-08-01</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -1603,7 +1603,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>01-09-2010</t>
+          <t>2010-09-01</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -1613,7 +1613,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>01-10-2010</t>
+          <t>2010-10-01</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -1623,7 +1623,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>01-11-2010</t>
+          <t>2010-11-01</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -1633,7 +1633,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>01-12-2010</t>
+          <t>2010-12-01</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -1643,7 +1643,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>01-01-2011</t>
+          <t>2011-01-01</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -1653,7 +1653,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>01-02-2011</t>
+          <t>2011-02-01</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -1663,7 +1663,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>01-03-2011</t>
+          <t>2011-03-01</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -1673,7 +1673,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>01-04-2011</t>
+          <t>2011-04-01</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -1683,7 +1683,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>01-05-2011</t>
+          <t>2011-05-01</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -1693,7 +1693,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>01-06-2011</t>
+          <t>2011-06-01</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -1703,7 +1703,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>01-07-2011</t>
+          <t>2011-07-01</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -1713,7 +1713,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>01-08-2011</t>
+          <t>2011-08-01</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -1723,7 +1723,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>01-09-2011</t>
+          <t>2011-09-01</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -1733,7 +1733,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>01-10-2011</t>
+          <t>2011-10-01</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -1743,7 +1743,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>01-11-2011</t>
+          <t>2011-11-01</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -1753,7 +1753,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>01-12-2011</t>
+          <t>2011-12-01</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -1763,7 +1763,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>01-01-2012</t>
+          <t>2012-01-01</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -1773,7 +1773,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>01-02-2012</t>
+          <t>2012-02-01</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -1783,7 +1783,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>01-03-2012</t>
+          <t>2012-03-01</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -1793,7 +1793,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>01-04-2012</t>
+          <t>2012-04-01</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -1803,7 +1803,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>01-05-2012</t>
+          <t>2012-05-01</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -1813,7 +1813,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>01-06-2012</t>
+          <t>2012-06-01</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -1823,7 +1823,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>01-07-2012</t>
+          <t>2012-07-01</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -1833,7 +1833,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>01-08-2012</t>
+          <t>2012-08-01</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -1843,7 +1843,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>01-09-2012</t>
+          <t>2012-09-01</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -1853,7 +1853,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>01-10-2012</t>
+          <t>2012-10-01</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -1863,7 +1863,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>01-11-2012</t>
+          <t>2012-11-01</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -1873,7 +1873,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>01-12-2012</t>
+          <t>2012-12-01</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -1883,7 +1883,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>01-01-2013</t>
+          <t>2013-01-01</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -1893,7 +1893,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>01-02-2013</t>
+          <t>2013-02-01</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -1903,7 +1903,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>01-03-2013</t>
+          <t>2013-03-01</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -1913,7 +1913,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>01-04-2013</t>
+          <t>2013-04-01</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -1923,7 +1923,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>01-05-2013</t>
+          <t>2013-05-01</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -1933,7 +1933,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>01-06-2013</t>
+          <t>2013-06-01</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -1943,7 +1943,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>01-07-2013</t>
+          <t>2013-07-01</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -1953,7 +1953,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>01-08-2013</t>
+          <t>2013-08-01</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -1963,7 +1963,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>01-09-2013</t>
+          <t>2013-09-01</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -1973,7 +1973,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>01-10-2013</t>
+          <t>2013-10-01</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -1983,7 +1983,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>01-11-2013</t>
+          <t>2013-11-01</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -1993,7 +1993,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>01-12-2013</t>
+          <t>2013-12-01</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -2003,7 +2003,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>01-01-2014</t>
+          <t>2014-01-01</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2013,7 +2013,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>01-02-2014</t>
+          <t>2014-02-01</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2023,7 +2023,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>01-03-2014</t>
+          <t>2014-03-01</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2033,7 +2033,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>01-04-2014</t>
+          <t>2014-04-01</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -2043,7 +2043,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>01-05-2014</t>
+          <t>2014-05-01</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -2053,7 +2053,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>01-06-2014</t>
+          <t>2014-06-01</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -2063,7 +2063,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>01-07-2014</t>
+          <t>2014-07-01</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -2073,7 +2073,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>01-08-2014</t>
+          <t>2014-08-01</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -2083,7 +2083,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>01-09-2014</t>
+          <t>2014-09-01</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -2093,7 +2093,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>01-10-2014</t>
+          <t>2014-10-01</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -2103,7 +2103,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>01-11-2014</t>
+          <t>2014-11-01</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -2113,7 +2113,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>01-12-2014</t>
+          <t>2014-12-01</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -2123,7 +2123,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>01-01-2015</t>
+          <t>2015-01-01</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -2133,7 +2133,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>01-02-2015</t>
+          <t>2015-02-01</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -2143,7 +2143,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>01-03-2015</t>
+          <t>2015-03-01</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -2153,7 +2153,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>01-04-2015</t>
+          <t>2015-04-01</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -2163,7 +2163,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>01-05-2015</t>
+          <t>2015-05-01</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -2173,7 +2173,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>01-06-2015</t>
+          <t>2015-06-01</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -2183,7 +2183,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>01-07-2015</t>
+          <t>2015-07-01</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -2193,7 +2193,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>01-08-2015</t>
+          <t>2015-08-01</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -2203,7 +2203,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>01-09-2015</t>
+          <t>2015-09-01</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -2213,7 +2213,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>01-10-2015</t>
+          <t>2015-10-01</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -2223,7 +2223,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>01-11-2015</t>
+          <t>2015-11-01</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -2233,7 +2233,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>01-12-2015</t>
+          <t>2015-12-01</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -2243,7 +2243,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>01-01-2016</t>
+          <t>2016-01-01</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -2253,7 +2253,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>01-02-2016</t>
+          <t>2016-02-01</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -2263,7 +2263,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>01-03-2016</t>
+          <t>2016-03-01</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -2273,7 +2273,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>01-04-2016</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -2283,7 +2283,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>01-05-2016</t>
+          <t>2016-05-01</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -2293,7 +2293,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>01-06-2016</t>
+          <t>2016-06-01</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -2303,7 +2303,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>01-07-2016</t>
+          <t>2016-07-01</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -2313,7 +2313,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>01-08-2016</t>
+          <t>2016-08-01</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -2323,7 +2323,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>01-09-2016</t>
+          <t>2016-09-01</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -2333,7 +2333,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>01-10-2016</t>
+          <t>2016-10-01</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -2343,7 +2343,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>01-11-2016</t>
+          <t>2016-11-01</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -2353,7 +2353,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>01-12-2016</t>
+          <t>2016-12-01</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -2363,7 +2363,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>01-01-2017</t>
+          <t>2017-01-01</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -2373,7 +2373,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>01-02-2017</t>
+          <t>2017-02-01</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -2383,7 +2383,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>01-03-2017</t>
+          <t>2017-03-01</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -2393,7 +2393,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>01-04-2017</t>
+          <t>2017-04-01</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -2403,7 +2403,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>01-05-2017</t>
+          <t>2017-05-01</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -2413,7 +2413,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>01-06-2017</t>
+          <t>2017-06-01</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -2423,7 +2423,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>01-07-2017</t>
+          <t>2017-07-01</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -2433,7 +2433,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>01-08-2017</t>
+          <t>2017-08-01</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -2443,7 +2443,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>01-09-2017</t>
+          <t>2017-09-01</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -2453,7 +2453,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>01-10-2017</t>
+          <t>2017-10-01</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -2463,7 +2463,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>01-11-2017</t>
+          <t>2017-11-01</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -2473,7 +2473,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>01-12-2017</t>
+          <t>2017-12-01</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -2483,7 +2483,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>01-01-2018</t>
+          <t>2018-01-01</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -2493,7 +2493,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>01-02-2018</t>
+          <t>2018-02-01</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -2503,7 +2503,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>01-03-2018</t>
+          <t>2018-03-01</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -2513,7 +2513,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>01-04-2018</t>
+          <t>2018-04-01</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -2523,7 +2523,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>01-05-2018</t>
+          <t>2018-05-01</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -2533,7 +2533,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>01-06-2018</t>
+          <t>2018-06-01</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -2543,7 +2543,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>01-07-2018</t>
+          <t>2018-07-01</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -2553,7 +2553,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>01-08-2018</t>
+          <t>2018-08-01</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -2563,7 +2563,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>01-09-2018</t>
+          <t>2018-09-01</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -2573,7 +2573,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>01-10-2018</t>
+          <t>2018-10-01</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -2583,7 +2583,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>01-11-2018</t>
+          <t>2018-11-01</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -2593,7 +2593,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>01-12-2018</t>
+          <t>2018-12-01</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -2603,7 +2603,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>01-01-2019</t>
+          <t>2019-01-01</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -2613,7 +2613,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>01-02-2019</t>
+          <t>2019-02-01</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -2623,7 +2623,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>01-03-2019</t>
+          <t>2019-03-01</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -2633,7 +2633,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>01-04-2019</t>
+          <t>2019-04-01</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -2643,7 +2643,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>01-05-2019</t>
+          <t>2019-05-01</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -2653,7 +2653,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>01-06-2019</t>
+          <t>2019-06-01</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -2663,7 +2663,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>01-07-2019</t>
+          <t>2019-07-01</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -2673,7 +2673,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>01-08-2019</t>
+          <t>2019-08-01</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -2683,7 +2683,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>01-09-2019</t>
+          <t>2019-09-01</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -2693,7 +2693,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>01-10-2019</t>
+          <t>2019-10-01</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -2703,7 +2703,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>01-11-2019</t>
+          <t>2019-11-01</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -2713,7 +2713,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>01-12-2019</t>
+          <t>2019-12-01</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -2723,7 +2723,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>01-01-2020</t>
+          <t>2020-01-01</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -2733,7 +2733,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>01-02-2020</t>
+          <t>2020-02-01</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -2743,7 +2743,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>01-03-2020</t>
+          <t>2020-03-01</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -2753,7 +2753,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>01-04-2020</t>
+          <t>2020-04-01</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -2763,7 +2763,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>01-05-2020</t>
+          <t>2020-05-01</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -2773,7 +2773,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>01-06-2020</t>
+          <t>2020-06-01</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -2783,7 +2783,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>01-07-2020</t>
+          <t>2020-07-01</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -2793,7 +2793,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>01-08-2020</t>
+          <t>2020-08-01</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -2803,7 +2803,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>01-09-2020</t>
+          <t>2020-09-01</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -2813,7 +2813,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>01-10-2020</t>
+          <t>2020-10-01</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -2823,7 +2823,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>01-11-2020</t>
+          <t>2020-11-01</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -2833,7 +2833,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>01-12-2020</t>
+          <t>2020-12-01</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -2843,7 +2843,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>01-01-2021</t>
+          <t>2021-01-01</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -2853,7 +2853,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>01-02-2021</t>
+          <t>2021-02-01</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -2863,7 +2863,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>01-03-2021</t>
+          <t>2021-03-01</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -2873,7 +2873,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>01-04-2021</t>
+          <t>2021-04-01</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -2883,7 +2883,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>01-05-2021</t>
+          <t>2021-05-01</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -2893,7 +2893,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>01-06-2021</t>
+          <t>2021-06-01</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -2903,7 +2903,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>01-07-2021</t>
+          <t>2021-07-01</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -2913,7 +2913,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>01-08-2021</t>
+          <t>2021-08-01</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -2923,7 +2923,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>01-09-2021</t>
+          <t>2021-09-01</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -2933,7 +2933,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>01-10-2021</t>
+          <t>2021-10-01</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -2943,7 +2943,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>01-11-2021</t>
+          <t>2021-11-01</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -2953,7 +2953,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>01-12-2021</t>
+          <t>2021-12-01</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -2963,7 +2963,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>01-01-2022</t>
+          <t>2022-01-01</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -2973,7 +2973,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>01-02-2022</t>
+          <t>2022-02-01</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -2983,7 +2983,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>01-03-2022</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -2993,7 +2993,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>01-04-2022</t>
+          <t>2022-04-01</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -3003,7 +3003,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>01-05-2022</t>
+          <t>2022-05-01</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -3013,7 +3013,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>01-06-2022</t>
+          <t>2022-06-01</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -3023,7 +3023,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>01-07-2022</t>
+          <t>2022-07-01</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -3033,7 +3033,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>01-08-2022</t>
+          <t>2022-08-01</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -3043,7 +3043,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>01-09-2022</t>
+          <t>2022-09-01</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -3053,7 +3053,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>01-10-2022</t>
+          <t>2022-10-01</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -3063,7 +3063,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>01-11-2022</t>
+          <t>2022-11-01</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -3073,7 +3073,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>01-12-2022</t>
+          <t>2022-12-01</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -3083,7 +3083,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>01-01-2023</t>
+          <t>2023-01-01</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -3093,7 +3093,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>01-02-2023</t>
+          <t>2023-02-01</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -3103,7 +3103,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>01-03-2023</t>
+          <t>2023-03-01</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -3113,7 +3113,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>01-04-2023</t>
+          <t>2023-04-01</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -3123,7 +3123,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>01-05-2023</t>
+          <t>2023-05-01</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -3133,7 +3133,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>01-06-2023</t>
+          <t>2023-06-01</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -3143,7 +3143,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>01-07-2023</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -3153,7 +3153,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>01-08-2023</t>
+          <t>2023-08-01</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -3163,7 +3163,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>01-09-2023</t>
+          <t>2023-09-01</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -3173,7 +3173,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>01-10-2023</t>
+          <t>2023-10-01</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -3183,7 +3183,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>01-11-2023</t>
+          <t>2023-11-01</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -3193,7 +3193,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>01-12-2023</t>
+          <t>2023-12-01</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -3203,7 +3203,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>01-01-2024</t>
+          <t>2024-01-01</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -3213,7 +3213,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>01-02-2024</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -3223,7 +3223,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>01-03-2024</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -3233,7 +3233,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>01-04-2024</t>
+          <t>2024-04-01</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -3243,7 +3243,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>01-05-2024</t>
+          <t>2024-05-01</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -3253,7 +3253,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>01-06-2024</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -3263,7 +3263,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>01-07-2024</t>
+          <t>2024-07-01</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -3273,7 +3273,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>01-08-2024</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -3283,7 +3283,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>01-09-2024</t>
+          <t>2024-09-01</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -3293,7 +3293,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>01-10-2024</t>
+          <t>2024-10-01</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -3303,7 +3303,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>01-11-2024</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -3313,7 +3313,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>01-12-2024</t>
+          <t>2024-12-01</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -3323,7 +3323,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>01-01-2025</t>
+          <t>2025-01-01</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -3333,7 +3333,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>01-02-2025</t>
+          <t>2025-02-01</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -3343,7 +3343,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>01-03-2025</t>
+          <t>2025-03-01</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -3353,7 +3353,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>01-04-2025</t>
+          <t>2025-04-01</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -3363,7 +3363,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>01-05-2025</t>
+          <t>2025-05-01</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -3373,7 +3373,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>01-06-2025</t>
+          <t>2025-06-01</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -3383,7 +3383,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -3393,7 +3393,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -3403,7 +3403,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -3413,7 +3413,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>2025-10-01</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -3423,7 +3423,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>2025-11-01</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -3433,7 +3433,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -3443,7 +3443,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -3453,7 +3453,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -3463,7 +3463,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -3473,7 +3473,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>01-04-2026</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -3483,7 +3483,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>01-05-2026</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -3493,7 +3493,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>01-06-2026</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B307" t="n">

</xml_diff>